<commit_message>
pruebitas con deficit como data de entrada
</commit_message>
<xml_diff>
--- a/data/Escenarios_DCH/Costo_variable/Swap_variable_3estaciones_320kW/elmo_data.xlsx
+++ b/data/Escenarios_DCH/Costo_variable/Swap_variable_3estaciones_320kW/elmo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Escenarios_DCH\Costo_variable\Swap_variable_3estaciones_320kW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC784850-8872-4192-AAE2-0AC1CB83C66A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C53C1D-A0AA-4ED0-B009-FCB2B45A18D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4275" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>

</xml_diff>